<commit_message>
SAGA/generics use FE4 class stats; drop illogical FE5 RES; Leif SAGA=FE4
- Class top-level (= SAGA / generic resolution) set to the FE4 version's bases
  and caps, so generic units and SAGA mode use FE4 class stats (incl. FE4 RES).
- Zero RES in FE5 class blocks (Archer/Hero/LordSeliph/Mercenary/Sniper/
  Soldier/Swordfighter/Warrior) — FE5 has no RES (MAG is magic defense).
- Leif: SAGA now uses his FE4 base stats (top-level=FE4); FE5 form (weak
  22/4/...) moved to versions.FE5. Nanna already SAGA=FE4 (unchanged).
- Also propagated the Cavalier->real-name rename into tools/*.py generators.
- Regenerated class_proportions.json.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0173CjjXKMnsNm8AgUP3We9A
</commit_message>
<xml_diff>
--- a/docs/FE4_FE5_Class_Proportions.xlsx
+++ b/docs/FE4_FE5_Class_Proportions.xlsx
@@ -611,190 +611,188 @@
       <c r="Q2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="R2" s="3" t="n">
-        <v>1.5</v>
-      </c>
+      <c r="R2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Armour</t>
+          <t>ArcherKnight</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>2.333</v>
+      </c>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C3" s="3" t="n">
-        <v>2.25</v>
-      </c>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
-      <c r="F3" s="3" t="n"/>
+      <c r="F3" s="3" t="n">
+        <v>1.2</v>
+      </c>
       <c r="G3" s="3" t="n"/>
       <c r="H3" s="3" t="n">
-        <v>1.25</v>
+        <v>2</v>
       </c>
       <c r="I3" s="3" t="n"/>
       <c r="J3" s="3" t="n">
-        <v>2.094</v>
+        <v>1.618</v>
       </c>
       <c r="K3" s="3" t="n">
         <v>1</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>0.75</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>1</v>
+        <v>1.05</v>
       </c>
       <c r="O3" s="3" t="n">
-        <v>0.9</v>
+        <v>1.05</v>
       </c>
       <c r="P3" s="3" t="n">
         <v>1.5</v>
       </c>
       <c r="Q3" s="3" t="n">
-        <v>1.25</v>
+        <v>1.05</v>
       </c>
       <c r="R3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Bandit</t>
+          <t>Armour</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>1.591</v>
+        <v>2</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>1</v>
+        <v>2.25</v>
       </c>
       <c r="D4" s="3" t="n"/>
       <c r="E4" s="3" t="n"/>
       <c r="F4" s="3" t="n"/>
       <c r="G4" s="3" t="n"/>
       <c r="H4" s="3" t="n">
-        <v>1.667</v>
+        <v>1.25</v>
       </c>
       <c r="I4" s="3" t="n"/>
       <c r="J4" s="3" t="n">
-        <v>1.733</v>
+        <v>2.094</v>
       </c>
       <c r="K4" s="3" t="n">
         <v>1</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0.75</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="O4" s="3" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="P4" s="3" t="n">
         <v>1.5</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="R4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Bard</t>
+          <t>AxeKnight</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>1.875</v>
-      </c>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="3" t="n">
-        <v>7</v>
-      </c>
+        <v>1.5</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>2.333</v>
+      </c>
+      <c r="D5" s="3" t="n"/>
       <c r="E5" s="3" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F5" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G5" s="3" t="n"/>
+      <c r="H5" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="3" t="n"/>
       <c r="I5" s="3" t="n"/>
       <c r="J5" s="3" t="n">
-        <v>2.783</v>
+        <v>1.667</v>
       </c>
       <c r="K5" s="3" t="n">
         <v>1</v>
       </c>
       <c r="L5" s="3" t="n">
-        <v>0.75</v>
+        <v>1.1</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>1.1</v>
+        <v>0.75</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>1.1</v>
+        <v>1.05</v>
       </c>
       <c r="O5" s="3" t="n">
-        <v>1.25</v>
+        <v>1.05</v>
       </c>
       <c r="P5" s="3" t="n">
         <v>1.5</v>
       </c>
       <c r="Q5" s="3" t="n">
-        <v>0.9</v>
+        <v>1.05</v>
       </c>
       <c r="R5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Baron</t>
+          <t>Bandit</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>1.731</v>
+        <v>1.591</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>2.333</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>1.167</v>
-      </c>
-      <c r="F6" s="3" t="n">
-        <v>2.333</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="D6" s="3" t="n"/>
+      <c r="E6" s="3" t="n"/>
+      <c r="F6" s="3" t="n"/>
       <c r="G6" s="3" t="n"/>
       <c r="H6" s="3" t="n">
-        <v>0.8</v>
+        <v>1.667</v>
       </c>
       <c r="I6" s="3" t="n"/>
       <c r="J6" s="3" t="n">
-        <v>1.54</v>
+        <v>1.733</v>
       </c>
       <c r="K6" s="3" t="n">
         <v>1</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>1.35</v>
+        <v>1</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>1.1</v>
+        <v>0.75</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>1.1</v>
+        <v>0.75</v>
       </c>
       <c r="O6" s="3" t="n">
         <v>1.1</v>
@@ -803,36 +801,34 @@
         <v>1.5</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>1.35</v>
+        <v>1</v>
       </c>
       <c r="R6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Bishop</t>
+          <t>Bard</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>1.75</v>
+        <v>1.875</v>
       </c>
       <c r="C7" s="3" t="n"/>
       <c r="D7" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F7" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="E7" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="F7" s="3" t="n">
-        <v>2.5</v>
-      </c>
       <c r="G7" s="3" t="n"/>
-      <c r="H7" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="H7" s="3" t="n"/>
       <c r="I7" s="3" t="n"/>
       <c r="J7" s="3" t="n">
-        <v>2.3</v>
+        <v>2.783</v>
       </c>
       <c r="K7" s="3" t="n">
         <v>1</v>
@@ -841,13 +837,13 @@
         <v>0.75</v>
       </c>
       <c r="M7" s="3" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="N7" s="3" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="O7" s="3" t="n">
         <v>1.25</v>
-      </c>
-      <c r="N7" s="3" t="n">
-        <v>1.15</v>
-      </c>
-      <c r="O7" s="3" t="n">
-        <v>1</v>
       </c>
       <c r="P7" s="3" t="n">
         <v>1.5</v>
@@ -860,159 +856,161 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>BowKnight</t>
+          <t>Baron</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>1.667</v>
+        <v>1.731</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>2</v>
+        <v>1.2</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>0</v>
+        <v>2.333</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>1.333</v>
+        <v>1.167</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>1.143</v>
+        <v>2.333</v>
       </c>
       <c r="G8" s="3" t="n"/>
       <c r="H8" s="3" t="n">
-        <v>1.6</v>
+        <v>0.8</v>
       </c>
       <c r="I8" s="3" t="n"/>
       <c r="J8" s="3" t="n">
-        <v>1.604</v>
+        <v>1.54</v>
       </c>
       <c r="K8" s="3" t="n">
         <v>1</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>1.25</v>
+        <v>1.35</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>0.75</v>
+        <v>1.1</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="P8" s="3" t="n">
         <v>1.5</v>
       </c>
       <c r="Q8" s="3" t="n">
-        <v>1.15</v>
+        <v>1.35</v>
       </c>
       <c r="R8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Cavalier</t>
+          <t>Bishop</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>2.333</v>
-      </c>
-      <c r="D9" s="3" t="n"/>
+        <v>1.75</v>
+      </c>
+      <c r="C9" s="3" t="n"/>
+      <c r="D9" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="E9" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="G9" s="3" t="n"/>
       <c r="H9" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I9" s="3" t="n"/>
       <c r="J9" s="3" t="n">
-        <v>1.667</v>
+        <v>2.3</v>
       </c>
       <c r="K9" s="3" t="n">
         <v>1</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>1.1</v>
+        <v>0.75</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>1.05</v>
+        <v>1.15</v>
       </c>
       <c r="O9" s="3" t="n">
-        <v>1.05</v>
+        <v>1</v>
       </c>
       <c r="P9" s="3" t="n">
         <v>1.5</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>1.05</v>
+        <v>0.9</v>
       </c>
       <c r="R9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>CavalierA</t>
+          <t>BowKnight</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>1.5</v>
+        <v>1.667</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>2.333</v>
-      </c>
-      <c r="D10" s="3" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="E10" s="3" t="n">
-        <v>2</v>
+        <v>1.333</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>1.5</v>
+        <v>1.143</v>
       </c>
       <c r="G10" s="3" t="n"/>
       <c r="H10" s="3" t="n">
-        <v>2</v>
+        <v>1.6</v>
       </c>
       <c r="I10" s="3" t="n"/>
       <c r="J10" s="3" t="n">
-        <v>1.667</v>
+        <v>1.604</v>
       </c>
       <c r="K10" s="3" t="n">
         <v>1</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>1.1</v>
+        <v>1.25</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0.75</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>1.05</v>
+        <v>1.15</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>1.05</v>
+        <v>1.15</v>
       </c>
       <c r="P10" s="3" t="n">
         <v>1.5</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>1.05</v>
+        <v>1.15</v>
       </c>
       <c r="R10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>CavalierB</t>
+          <t>Cavalier</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
@@ -1026,7 +1024,7 @@
         <v>2</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="G11" s="3" t="n"/>
       <c r="H11" s="3" t="n">
@@ -1034,7 +1032,7 @@
       </c>
       <c r="I11" s="3" t="n"/>
       <c r="J11" s="3" t="n">
-        <v>1.618</v>
+        <v>1.667</v>
       </c>
       <c r="K11" s="3" t="n">
         <v>1</v>
@@ -1062,121 +1060,115 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>CavalierL</t>
+          <t>Citizen</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="C12" s="3" t="n">
-        <v>2.333</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="C12" s="3" t="n"/>
       <c r="D12" s="3" t="n"/>
-      <c r="E12" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F12" s="3" t="n">
-        <v>1.5</v>
-      </c>
+      <c r="E12" s="3" t="n"/>
+      <c r="F12" s="3" t="n"/>
       <c r="G12" s="3" t="n"/>
-      <c r="H12" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="H12" s="3" t="n"/>
       <c r="I12" s="3" t="n"/>
       <c r="J12" s="3" t="n">
-        <v>1.667</v>
+        <v>3.2</v>
       </c>
       <c r="K12" s="3" t="n">
         <v>1</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>1.1</v>
+        <v>0.75</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0.75</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>1.05</v>
+        <v>0.75</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>1.05</v>
+        <v>1.25</v>
       </c>
       <c r="P12" s="3" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>1.05</v>
+        <v>0.85</v>
       </c>
       <c r="R12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>CavalierS</t>
+          <t>Dancer</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="C13" s="3" t="n">
-        <v>2.333</v>
-      </c>
+        <v>1.857</v>
+      </c>
+      <c r="C13" s="3" t="n"/>
       <c r="D13" s="3" t="n"/>
-      <c r="E13" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E13" s="3" t="n"/>
       <c r="F13" s="3" t="n">
-        <v>1.5</v>
+        <v>3.5</v>
       </c>
       <c r="G13" s="3" t="n"/>
-      <c r="H13" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="H13" s="3" t="n"/>
       <c r="I13" s="3" t="n"/>
       <c r="J13" s="3" t="n">
-        <v>1.667</v>
+        <v>2.562</v>
       </c>
       <c r="K13" s="3" t="n">
         <v>1</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0.75</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>1.05</v>
+        <v>0.8</v>
       </c>
       <c r="O13" s="3" t="n">
-        <v>1.05</v>
+        <v>1.1</v>
       </c>
       <c r="P13" s="3" t="n">
         <v>1.5</v>
       </c>
       <c r="Q13" s="3" t="n">
-        <v>1.05</v>
+        <v>0.8</v>
       </c>
       <c r="R13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Citizen</t>
+          <t>DarkBishop</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>2</v>
+        <v>1.333</v>
       </c>
       <c r="C14" s="3" t="n"/>
-      <c r="D14" s="3" t="n"/>
-      <c r="E14" s="3" t="n"/>
-      <c r="F14" s="3" t="n"/>
+      <c r="D14" s="3" t="n">
+        <v>1.667</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>1.667</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>1.667</v>
+      </c>
       <c r="G14" s="3" t="n"/>
-      <c r="H14" s="3" t="n"/>
+      <c r="H14" s="3" t="n">
+        <v>1.667</v>
+      </c>
       <c r="I14" s="3" t="n"/>
       <c r="J14" s="3" t="n">
-        <v>3.2</v>
+        <v>1.702</v>
       </c>
       <c r="K14" s="3" t="n">
         <v>1</v>
@@ -1185,10 +1177,10 @@
         <v>0.75</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>0.75</v>
+        <v>1.5</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="O14" s="3" t="n">
         <v>1.25</v>
@@ -1197,80 +1189,86 @@
         <v>1.5</v>
       </c>
       <c r="Q14" s="3" t="n">
-        <v>0.85</v>
+        <v>1.25</v>
       </c>
       <c r="R14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Dancer</t>
+          <t>DarkMage</t>
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>1.857</v>
+        <v>1.667</v>
       </c>
       <c r="C15" s="3" t="n"/>
-      <c r="D15" s="3" t="n"/>
-      <c r="E15" s="3" t="n"/>
+      <c r="D15" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F15" s="3" t="n">
-        <v>3.5</v>
+        <v>2.667</v>
       </c>
       <c r="G15" s="3" t="n"/>
-      <c r="H15" s="3" t="n"/>
+      <c r="H15" s="3" t="n">
+        <v>1.75</v>
+      </c>
       <c r="I15" s="3" t="n"/>
       <c r="J15" s="3" t="n">
-        <v>2.562</v>
+        <v>2.075</v>
       </c>
       <c r="K15" s="3" t="n">
         <v>1</v>
       </c>
       <c r="L15" s="3" t="n">
-        <v>0.9</v>
+        <v>0.75</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>0.8</v>
+        <v>1.15</v>
       </c>
       <c r="O15" s="3" t="n">
-        <v>1.1</v>
+        <v>1.15</v>
       </c>
       <c r="P15" s="3" t="n">
         <v>1.5</v>
       </c>
       <c r="Q15" s="3" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
       <c r="R15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>DarkBishop</t>
+          <t>DarkPrince</t>
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>1.333</v>
+        <v>0.6</v>
       </c>
       <c r="C16" s="3" t="n"/>
       <c r="D16" s="3" t="n">
-        <v>1.667</v>
+        <v>0.75</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>1.667</v>
+        <v>0.6</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>1.667</v>
+        <v>0.6</v>
       </c>
       <c r="G16" s="3" t="n"/>
       <c r="H16" s="3" t="n">
-        <v>1.667</v>
+        <v>0.5</v>
       </c>
       <c r="I16" s="3" t="n"/>
       <c r="J16" s="3" t="n">
-        <v>1.702</v>
+        <v>0.723</v>
       </c>
       <c r="K16" s="3" t="n">
         <v>1</v>
@@ -1282,10 +1280,10 @@
         <v>1.5</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>1.25</v>
+        <v>1.35</v>
       </c>
       <c r="O16" s="3" t="n">
-        <v>1.25</v>
+        <v>1.35</v>
       </c>
       <c r="P16" s="3" t="n">
         <v>1.5</v>
@@ -1298,137 +1296,137 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>DarkMage</t>
+          <t>DragonKnight</t>
         </is>
       </c>
       <c r="B17" s="3" t="n">
         <v>1.667</v>
       </c>
-      <c r="C17" s="3" t="n"/>
+      <c r="C17" s="3" t="n">
+        <v>1.429</v>
+      </c>
       <c r="D17" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>2</v>
+        <v>1.167</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>2.667</v>
+        <v>1</v>
       </c>
       <c r="G17" s="3" t="n"/>
       <c r="H17" s="3" t="n">
-        <v>1.75</v>
+        <v>1.222</v>
       </c>
       <c r="I17" s="3" t="n"/>
       <c r="J17" s="3" t="n">
-        <v>2.075</v>
+        <v>1.396</v>
       </c>
       <c r="K17" s="3" t="n">
         <v>1</v>
       </c>
       <c r="L17" s="3" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>1.25</v>
+        <v>0.75</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="O17" s="3" t="n">
-        <v>1.15</v>
+        <v>1.05</v>
       </c>
       <c r="P17" s="3" t="n">
         <v>1.5</v>
       </c>
       <c r="Q17" s="3" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>DarkPrince</t>
+          <t>DragonRider</t>
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="C18" s="3" t="n"/>
-      <c r="D18" s="3" t="n">
-        <v>0.75</v>
-      </c>
+        <v>2.188</v>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="D18" s="3" t="n"/>
       <c r="E18" s="3" t="n">
-        <v>0.6</v>
+        <v>1.667</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>0.6</v>
+        <v>1.25</v>
       </c>
       <c r="G18" s="3" t="n"/>
       <c r="H18" s="3" t="n">
-        <v>0.5</v>
+        <v>1.143</v>
       </c>
       <c r="I18" s="3" t="n"/>
       <c r="J18" s="3" t="n">
-        <v>0.723</v>
+        <v>1.771</v>
       </c>
       <c r="K18" s="3" t="n">
         <v>1</v>
       </c>
       <c r="L18" s="3" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>1.5</v>
+        <v>0.75</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>1.35</v>
+        <v>1.1</v>
       </c>
       <c r="O18" s="3" t="n">
-        <v>1.35</v>
+        <v>1.05</v>
       </c>
       <c r="P18" s="3" t="n">
         <v>1.5</v>
       </c>
       <c r="Q18" s="3" t="n">
-        <v>1.25</v>
+        <v>1.3</v>
       </c>
       <c r="R18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>DragonKnight</t>
+          <t>DukeKnight</t>
         </is>
       </c>
       <c r="B19" s="3" t="n">
         <v>1.667</v>
       </c>
       <c r="C19" s="3" t="n">
-        <v>1.429</v>
-      </c>
-      <c r="D19" s="3" t="n">
-        <v>0</v>
-      </c>
+        <v>2.4</v>
+      </c>
+      <c r="D19" s="3" t="n"/>
       <c r="E19" s="3" t="n">
         <v>1.167</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>1</v>
+        <v>1.167</v>
       </c>
       <c r="G19" s="3" t="n"/>
       <c r="H19" s="3" t="n">
-        <v>1.222</v>
+        <v>1.6</v>
       </c>
       <c r="I19" s="3" t="n"/>
       <c r="J19" s="3" t="n">
-        <v>1.396</v>
+        <v>1.674</v>
       </c>
       <c r="K19" s="3" t="n">
         <v>1</v>
       </c>
       <c r="L19" s="3" t="n">
-        <v>1.25</v>
+        <v>1.35</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0.75</v>
@@ -1437,196 +1435,196 @@
         <v>1.1</v>
       </c>
       <c r="O19" s="3" t="n">
-        <v>1.05</v>
+        <v>1.1</v>
       </c>
       <c r="P19" s="3" t="n">
         <v>1.5</v>
       </c>
       <c r="Q19" s="3" t="n">
-        <v>1.3</v>
+        <v>1.15</v>
       </c>
       <c r="R19" s="3" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>DragonRider</t>
+          <t>Emperor</t>
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>2.188</v>
+        <v>1.731</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="D20" s="3" t="n"/>
+        <v>2.143</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>15</v>
+      </c>
       <c r="E20" s="3" t="n">
-        <v>1.667</v>
+        <v>3</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>1.25</v>
+        <v>7.5</v>
       </c>
       <c r="G20" s="3" t="n"/>
       <c r="H20" s="3" t="n">
-        <v>1.143</v>
+        <v>1.25</v>
       </c>
       <c r="I20" s="3" t="n"/>
       <c r="J20" s="3" t="n">
-        <v>1.771</v>
+        <v>2.547</v>
       </c>
       <c r="K20" s="3" t="n">
         <v>1</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>1.25</v>
+        <v>1.5</v>
       </c>
       <c r="M20" s="3" t="n">
-        <v>0.75</v>
+        <v>1.5</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>1.1</v>
+        <v>1.5</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>1.05</v>
+        <v>1.5</v>
       </c>
       <c r="P20" s="3" t="n">
         <v>1.5</v>
       </c>
       <c r="Q20" s="3" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="R20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>DukeKnight</t>
+          <t>FalconKnight</t>
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>1.667</v>
+        <v>2</v>
       </c>
       <c r="C21" s="3" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="D21" s="3" t="n"/>
+        <v>1.167</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="E21" s="3" t="n">
-        <v>1.167</v>
+        <v>1.714</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>1.167</v>
+        <v>1.5</v>
       </c>
       <c r="G21" s="3" t="n"/>
       <c r="H21" s="3" t="n">
-        <v>1.6</v>
+        <v>1.2</v>
       </c>
       <c r="I21" s="3" t="n"/>
       <c r="J21" s="3" t="n">
-        <v>1.674</v>
+        <v>1.8</v>
       </c>
       <c r="K21" s="3" t="n">
         <v>1</v>
       </c>
       <c r="L21" s="3" t="n">
-        <v>1.35</v>
+        <v>1.1</v>
       </c>
       <c r="M21" s="3" t="n">
-        <v>0.75</v>
+        <v>1.1</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>1.1</v>
+        <v>1.25</v>
       </c>
       <c r="O21" s="3" t="n">
-        <v>1.1</v>
+        <v>1.5</v>
       </c>
       <c r="P21" s="3" t="n">
         <v>1.5</v>
       </c>
       <c r="Q21" s="3" t="n">
-        <v>1.15</v>
+        <v>1.05</v>
       </c>
       <c r="R21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Emperor</t>
+          <t>Fighter</t>
         </is>
       </c>
       <c r="B22" s="3" t="n">
-        <v>1.731</v>
+        <v>1.75</v>
       </c>
       <c r="C22" s="3" t="n">
-        <v>2.143</v>
-      </c>
-      <c r="D22" s="3" t="n">
-        <v>15</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="D22" s="3" t="n"/>
       <c r="E22" s="3" t="n">
-        <v>3</v>
+        <v>0.75</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>7.5</v>
+        <v>2</v>
       </c>
       <c r="G22" s="3" t="n"/>
       <c r="H22" s="3" t="n">
-        <v>1.25</v>
+        <v>4</v>
       </c>
       <c r="I22" s="3" t="n"/>
       <c r="J22" s="3" t="n">
-        <v>2.547</v>
+        <v>1.829</v>
       </c>
       <c r="K22" s="3" t="n">
         <v>1</v>
       </c>
       <c r="L22" s="3" t="n">
-        <v>1.5</v>
+        <v>1.15</v>
       </c>
       <c r="M22" s="3" t="n">
-        <v>1.5</v>
+        <v>0.75</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>1.5</v>
+        <v>0.9</v>
       </c>
       <c r="O22" s="3" t="n">
-        <v>1.5</v>
+        <v>1.25</v>
       </c>
       <c r="P22" s="3" t="n">
         <v>1.5</v>
       </c>
       <c r="Q22" s="3" t="n">
-        <v>1.5</v>
+        <v>1.15</v>
       </c>
       <c r="R22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>FalconKnight</t>
+          <t>FreeKnight</t>
         </is>
       </c>
       <c r="B23" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C23" s="3" t="n">
+        <v>2.333</v>
+      </c>
+      <c r="D23" s="3" t="n"/>
+      <c r="E23" s="3" t="n">
         <v>2</v>
-      </c>
-      <c r="C23" s="3" t="n">
-        <v>1.167</v>
-      </c>
-      <c r="D23" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" s="3" t="n">
-        <v>1.714</v>
       </c>
       <c r="F23" s="3" t="n">
         <v>1.5</v>
       </c>
       <c r="G23" s="3" t="n"/>
       <c r="H23" s="3" t="n">
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="I23" s="3" t="n"/>
       <c r="J23" s="3" t="n">
-        <v>1.8</v>
+        <v>1.667</v>
       </c>
       <c r="K23" s="3" t="n">
         <v>1</v>
@@ -1635,13 +1633,13 @@
         <v>1.1</v>
       </c>
       <c r="M23" s="3" t="n">
-        <v>1.1</v>
+        <v>0.75</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>1.25</v>
+        <v>1.05</v>
       </c>
       <c r="O23" s="3" t="n">
-        <v>1.5</v>
+        <v>1.05</v>
       </c>
       <c r="P23" s="3" t="n">
         <v>1.5</v>
@@ -1654,133 +1652,135 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Fighter</t>
+          <t>General</t>
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>1.75</v>
+        <v>1.538</v>
       </c>
       <c r="C24" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D24" s="3" t="n"/>
+        <v>1.429</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="E24" s="3" t="n">
-        <v>0.75</v>
+        <v>1.2</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="G24" s="3" t="n"/>
       <c r="H24" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I24" s="3" t="n"/>
       <c r="J24" s="3" t="n">
-        <v>1.829</v>
+        <v>1.434</v>
       </c>
       <c r="K24" s="3" t="n">
         <v>1</v>
       </c>
       <c r="L24" s="3" t="n">
-        <v>1.15</v>
+        <v>1.25</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0.75</v>
       </c>
       <c r="N24" s="3" t="n">
-        <v>0.9</v>
+        <v>1.05</v>
       </c>
       <c r="O24" s="3" t="n">
-        <v>1.25</v>
+        <v>1</v>
       </c>
       <c r="P24" s="3" t="n">
         <v>1.5</v>
       </c>
       <c r="Q24" s="3" t="n">
-        <v>1.15</v>
+        <v>1.35</v>
       </c>
       <c r="R24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>GreatKnight</t>
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>1.538</v>
+        <v>1.667</v>
       </c>
       <c r="C25" s="3" t="n">
-        <v>1.429</v>
+        <v>2.4</v>
       </c>
       <c r="D25" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>1.2</v>
+        <v>1.167</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>2.5</v>
+        <v>1.167</v>
       </c>
       <c r="G25" s="3" t="n"/>
       <c r="H25" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I25" s="3" t="n"/>
       <c r="J25" s="3" t="n">
-        <v>1.434</v>
+        <v>1.681</v>
       </c>
       <c r="K25" s="3" t="n">
         <v>1</v>
       </c>
       <c r="L25" s="3" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="M25" s="3" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="N25" s="3" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="O25" s="3" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="P25" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Q25" s="3" t="n">
         <v>1.25</v>
-      </c>
-      <c r="M25" s="3" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="N25" s="3" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="O25" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="P25" s="3" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="Q25" s="3" t="n">
-        <v>1.35</v>
       </c>
       <c r="R25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>GreatKnight</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="B26" s="3" t="n">
         <v>1.667</v>
       </c>
       <c r="C26" s="3" t="n">
-        <v>2.4</v>
+        <v>2</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>1.167</v>
+        <v>1.714</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>1.167</v>
+        <v>1.333</v>
       </c>
       <c r="G26" s="3" t="n"/>
       <c r="H26" s="3" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="I26" s="3" t="n"/>
       <c r="J26" s="3" t="n">
-        <v>1.681</v>
+        <v>1.712</v>
       </c>
       <c r="K26" s="3" t="n">
         <v>1</v>
@@ -1789,80 +1789,76 @@
         <v>1.35</v>
       </c>
       <c r="M26" s="3" t="n">
-        <v>0.75</v>
+        <v>0.9</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>1.1</v>
+        <v>1.35</v>
       </c>
       <c r="O26" s="3" t="n">
-        <v>1.1</v>
+        <v>1.35</v>
       </c>
       <c r="P26" s="3" t="n">
         <v>1.5</v>
       </c>
       <c r="Q26" s="3" t="n">
-        <v>1.25</v>
+        <v>1.1</v>
       </c>
       <c r="R26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>HighPriest</t>
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>1.667</v>
-      </c>
-      <c r="C27" s="3" t="n">
+        <v>1.944</v>
+      </c>
+      <c r="C27" s="3" t="n"/>
+      <c r="D27" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="D27" s="3" t="n">
+      <c r="E27" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E27" s="3" t="n">
-        <v>1.714</v>
-      </c>
       <c r="F27" s="3" t="n">
-        <v>1.333</v>
+        <v>2.667</v>
       </c>
       <c r="G27" s="3" t="n"/>
       <c r="H27" s="3" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="I27" s="3" t="n">
-        <v>0.5</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="I27" s="3" t="n"/>
       <c r="J27" s="3" t="n">
-        <v>1.534</v>
+        <v>2.419</v>
       </c>
       <c r="K27" s="3" t="n">
         <v>1</v>
       </c>
       <c r="L27" s="3" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="M27" s="3" t="n">
         <v>1.35</v>
       </c>
-      <c r="M27" s="3" t="n">
+      <c r="N27" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="O27" s="3" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="P27" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Q27" s="3" t="n">
         <v>0.9</v>
-      </c>
-      <c r="N27" s="3" t="n">
-        <v>1.35</v>
-      </c>
-      <c r="O27" s="3" t="n">
-        <v>1.35</v>
-      </c>
-      <c r="P27" s="3" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="Q27" s="3" t="n">
-        <v>1.1</v>
       </c>
       <c r="R27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>HighPriest</t>
+          <t>HighPriestess</t>
         </is>
       </c>
       <c r="B28" s="3" t="n">
@@ -1912,50 +1908,50 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>HighPriestess</t>
+          <t>LanceKnight</t>
         </is>
       </c>
       <c r="B29" s="3" t="n">
-        <v>1.944</v>
-      </c>
-      <c r="C29" s="3" t="n"/>
-      <c r="D29" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C29" s="3" t="n">
+        <v>2.333</v>
+      </c>
+      <c r="D29" s="3" t="n"/>
+      <c r="E29" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="E29" s="3" t="n">
-        <v>3</v>
-      </c>
       <c r="F29" s="3" t="n">
-        <v>2.667</v>
+        <v>1.5</v>
       </c>
       <c r="G29" s="3" t="n"/>
       <c r="H29" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I29" s="3" t="n"/>
       <c r="J29" s="3" t="n">
-        <v>2.419</v>
+        <v>1.667</v>
       </c>
       <c r="K29" s="3" t="n">
         <v>1</v>
       </c>
       <c r="L29" s="3" t="n">
-        <v>0.75</v>
+        <v>1.1</v>
       </c>
       <c r="M29" s="3" t="n">
-        <v>1.35</v>
+        <v>0.75</v>
       </c>
       <c r="N29" s="3" t="n">
-        <v>1.2</v>
+        <v>1.05</v>
       </c>
       <c r="O29" s="3" t="n">
-        <v>1.15</v>
+        <v>1.05</v>
       </c>
       <c r="P29" s="3" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="Q29" s="3" t="n">
-        <v>0.9</v>
+        <v>1.05</v>
       </c>
       <c r="R29" s="3" t="n"/>
     </row>
@@ -2159,9 +2155,7 @@
       <c r="Q33" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="R33" s="3" t="n">
-        <v>0.75</v>
-      </c>
+      <c r="R33" s="3" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2286,11 +2280,9 @@
       <c r="H36" s="3" t="n">
         <v>2.5</v>
       </c>
-      <c r="I36" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="I36" s="3" t="n"/>
       <c r="J36" s="3" t="n">
-        <v>1.476</v>
+        <v>1.722</v>
       </c>
       <c r="K36" s="3" t="n">
         <v>1</v>
@@ -2313,9 +2305,7 @@
       <c r="Q36" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="R36" s="3" t="n">
-        <v>2.5</v>
-      </c>
+      <c r="R36" s="3" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2794,11 +2784,9 @@
       <c r="H46" s="3" t="n">
         <v>2.333</v>
       </c>
-      <c r="I46" s="3" t="n">
-        <v>0.429</v>
-      </c>
+      <c r="I46" s="3" t="n"/>
       <c r="J46" s="3" t="n">
-        <v>1.654</v>
+        <v>1.911</v>
       </c>
       <c r="K46" s="3" t="n">
         <v>1</v>
@@ -2867,9 +2855,7 @@
       <c r="Q47" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="R47" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="R47" s="3" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2894,11 +2880,9 @@
       <c r="H48" s="3" t="n">
         <v>2.5</v>
       </c>
-      <c r="I48" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="I48" s="3" t="n"/>
       <c r="J48" s="3" t="n">
-        <v>1.476</v>
+        <v>1.722</v>
       </c>
       <c r="K48" s="3" t="n">
         <v>1</v>
@@ -2921,9 +2905,7 @@
       <c r="Q48" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="R48" s="3" t="n">
-        <v>2.5</v>
-      </c>
+      <c r="R48" s="3" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3088,11 +3070,9 @@
       <c r="H52" s="3" t="n">
         <v>1.667</v>
       </c>
-      <c r="I52" s="3" t="n">
-        <v>0.5</v>
-      </c>
+      <c r="I52" s="3" t="n"/>
       <c r="J52" s="3" t="n">
-        <v>1.35</v>
+        <v>1.5</v>
       </c>
       <c r="K52" s="3" t="n">
         <v>1</v>

</xml_diff>